<commit_message>
feat: ByteCtrl RTL 구현 및 I2cMaster 골격 작성, BitCtrl SCL 주기 스펙 수정
- source/ByteCtrl.vhd: 2-process 스타일로 바이트 단위 송수신 FSM 신규 구현
  (LOAD/SHIFT_BIT/DONE, TxBit 출력 포트 승격)
- sim/ByteCtrlTb.vhd: ByteCtrl 단독 검증용 테스트벤치 작성
- source/I2cMaster.vhd: BitCtrl/ByteCtrl 형제 인스턴스화 배선 및 FSM 본체
  1차 작성 (IDLE~STOP, ByteStart/rw 세트 배선 진행 중)
- source/BitCtrl.vhd: T_LOW 65→90 수정, SCL 주기를 2.56us(≈390kHz)로
  맞춰 24LC256 Fast-mode(400kHz) 스펙 위반 해소
- sim/BitCtrlTb.vhd: START/STOP 조건 테스트 시나리오 추가
- 참고사항: I2cMaster/ByteData FSM drawio, 블록다이어그램, 타이밍 계산
  엑셀을 2계층 flat 구조(I2cMaster가 BitCtrl/ByteCtrl을 형제로 직접
  인스턴스화)로 갱신
- 참고사항/정리: 작업 로그를 정리 폴더로 이동, 9/9~9/11 일일 로그 추가

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/참고사항/SysClk_Timing_Calc.xlsx
+++ b/참고사항/SysClk_Timing_Calc.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="57">
   <si>
     <t>SysClk 타이밍 계산표</t>
   </si>
@@ -736,8 +736,9 @@
       <c r="D7" t="s">
         <v>16</v>
       </c>
-      <c r="E7" t="s">
-        <v>1</v>
+      <c r="E7">
+        <f>C7/20</f>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
         <v>1</v>
@@ -759,8 +760,9 @@
       <c r="D8" t="s">
         <v>19</v>
       </c>
-      <c r="E8" t="s">
-        <v>1</v>
+      <c r="E8">
+        <f t="shared" ref="E8:E20" si="0">C8/20</f>
+        <v>65</v>
       </c>
       <c r="F8" t="s">
         <v>1</v>
@@ -782,8 +784,9 @@
       <c r="D9" t="s">
         <v>22</v>
       </c>
-      <c r="E9" t="s">
-        <v>1</v>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="F9" t="s">
         <v>1</v>
@@ -805,8 +808,9 @@
       <c r="D10" t="s">
         <v>25</v>
       </c>
-      <c r="E10" t="s">
-        <v>1</v>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="F10" t="s">
         <v>1</v>
@@ -828,8 +832,9 @@
       <c r="D11" t="s">
         <v>28</v>
       </c>
-      <c r="E11" t="s">
-        <v>1</v>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="F11" t="s">
         <v>1</v>
@@ -851,8 +856,9 @@
       <c r="D12" t="s">
         <v>32</v>
       </c>
-      <c r="E12" t="s">
-        <v>1</v>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="F12" t="s">
         <v>1</v>
@@ -874,8 +880,9 @@
       <c r="D13" t="s">
         <v>36</v>
       </c>
-      <c r="E13" t="s">
-        <v>1</v>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="F13" t="s">
         <v>1</v>
@@ -897,14 +904,21 @@
       <c r="D14" t="s">
         <v>39</v>
       </c>
-      <c r="E14" t="s">
-        <v>1</v>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>65</v>
       </c>
       <c r="F14" t="s">
         <v>1</v>
       </c>
       <c r="G14" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -920,8 +934,9 @@
       <c r="D16" t="s">
         <v>1</v>
       </c>
-      <c r="E16" t="s">
-        <v>1</v>
+      <c r="E16" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
       </c>
       <c r="F16" t="s">
         <v>1</v>
@@ -943,8 +958,9 @@
       <c r="D17" t="s">
         <v>43</v>
       </c>
-      <c r="E17" t="s">
-        <v>1</v>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="F17" t="s">
         <v>1</v>
@@ -966,8 +982,9 @@
       <c r="D18" t="s">
         <v>43</v>
       </c>
-      <c r="E18" t="s">
-        <v>1</v>
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="F18" t="s">
         <v>1</v>
@@ -989,8 +1006,9 @@
       <c r="D19" t="s">
         <v>49</v>
       </c>
-      <c r="E19" t="s">
-        <v>1</v>
+      <c r="E19">
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
       <c r="F19" t="s">
         <v>1</v>
@@ -1012,8 +1030,9 @@
       <c r="D20" t="s">
         <v>54</v>
       </c>
-      <c r="E20" t="s">
-        <v>1</v>
+      <c r="E20" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
       </c>
       <c r="F20" t="s">
         <v>1</v>
@@ -1025,9 +1044,10 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G5 A8:G20 B7:G7 A6:E6 G6" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G5 A15:D20 B7:D7 A6:E6 G6 F7:G7 A8:D14 F8:G14 F15:G20" numberStoredAsText="1"/>
   </ignoredErrors>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>